<commit_message>
Update BOM and iBOM
Minor changes to component package sizes and values.
</commit_message>
<xml_diff>
--- a/BOM/NCC_Blackbird_PoC_BOM_verB_013.xlsx
+++ b/BOM/NCC_Blackbird_PoC_BOM_verB_013.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1210" uniqueCount="592">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1220" uniqueCount="599">
   <si>
     <t xml:space="preserve">MME P/N</t>
   </si>
@@ -733,10 +733,10 @@
     <t xml:space="preserve">C10</t>
   </si>
   <si>
-    <t xml:space="preserve">GRM1885C1H162JA01D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">490-1456-1-ND</t>
+    <t xml:space="preserve">C0805C162J5GACTU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">399-C0805C162J5GACTUCT-ND</t>
   </si>
   <si>
     <t xml:space="preserve">Cap, ceramic, 0.12uF, 50V, 10%, X7R, SMT 0805</t>
@@ -745,13 +745,10 @@
     <t xml:space="preserve">C11</t>
   </si>
   <si>
-    <t xml:space="preserve">Cal-Chip Electronics, Inc.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GMC21X7R123K50NT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4713-GMC21X7R123K50NTCT-ND</t>
+    <t xml:space="preserve">CC0805KRX7R9BB124</t>
+  </si>
+  <si>
+    <t xml:space="preserve">311-4323-1-ND</t>
   </si>
   <si>
     <t xml:space="preserve">Cap, ceramic, 0.01uF, 50V, 5%, NP0, SMT 0805</t>
@@ -823,10 +820,10 @@
     <t xml:space="preserve">C36</t>
   </si>
   <si>
-    <t xml:space="preserve">C0603C394J4RACTU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">399-C0603C394J4RACTUCT-ND</t>
+    <t xml:space="preserve">0805YC394JAT2A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">478-10574-1-ND</t>
   </si>
   <si>
     <t xml:space="preserve">Cap, ceramic, 5.6nF, 50V, 5%, NP0, SMT 0805</t>
@@ -1282,6 +1279,12 @@
     <t xml:space="preserve">846-LTR100JZPJ160CT-ND</t>
   </si>
   <si>
+    <t xml:space="preserve">TE Connectivity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3430A3F16RTDF</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resistor, 30.1K, 1%, SMD 0805</t>
   </si>
   <si>
@@ -1823,6 +1826,24 @@
   </si>
   <si>
     <t xml:space="preserve">Total Cost =</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Small O-ring</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1174N781</t>
+  </si>
+  <si>
+    <t xml:space="preserve">old</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1174N422</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Large O-ring</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1302N155</t>
   </si>
   <si>
     <t xml:space="preserve">Future Components</t>
@@ -6962,7 +6983,7 @@
         <v>27</v>
       </c>
       <c r="I77" s="22" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="J77" s="22" t="s">
         <v>227</v>
@@ -6978,18 +6999,18 @@
       <c r="O77" s="17"/>
       <c r="P77" s="17"/>
       <c r="Q77" s="15" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="R77" s="34" t="n">
         <f aca="false">(F77*Q77)</f>
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="S77" s="15" t="n">
-        <v>0.043</v>
+        <v>0.303</v>
       </c>
       <c r="T77" s="35" t="n">
         <f aca="false">(F77*S77)</f>
-        <v>0.043</v>
+        <v>0.303</v>
       </c>
       <c r="U77" s="17"/>
     </row>
@@ -7013,16 +7034,16 @@
         <v>27</v>
       </c>
       <c r="I78" s="22" t="s">
+        <v>209</v>
+      </c>
+      <c r="J78" s="22" t="s">
         <v>231</v>
-      </c>
-      <c r="J78" s="22" t="s">
-        <v>232</v>
       </c>
       <c r="K78" s="22" t="s">
         <v>32</v>
       </c>
       <c r="L78" s="22" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="M78" s="17"/>
       <c r="N78" s="17"/>
@@ -7049,10 +7070,10 @@
       <c r="B79" s="17"/>
       <c r="C79" s="17"/>
       <c r="D79" s="17" t="s">
+        <v>233</v>
+      </c>
+      <c r="E79" s="17" t="s">
         <v>234</v>
-      </c>
-      <c r="E79" s="17" t="s">
-        <v>235</v>
       </c>
       <c r="F79" s="32" t="n">
         <v>1</v>
@@ -7064,16 +7085,16 @@
         <v>27</v>
       </c>
       <c r="I79" s="17" t="s">
+        <v>235</v>
+      </c>
+      <c r="J79" s="17" t="s">
         <v>236</v>
-      </c>
-      <c r="J79" s="17" t="s">
-        <v>237</v>
       </c>
       <c r="K79" s="17" t="s">
         <v>32</v>
       </c>
       <c r="L79" s="17" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="M79" s="17"/>
       <c r="N79" s="17"/>
@@ -7335,10 +7356,10 @@
       <c r="B80" s="20"/>
       <c r="C80" s="17"/>
       <c r="D80" s="22" t="s">
+        <v>238</v>
+      </c>
+      <c r="E80" s="17" t="s">
         <v>239</v>
-      </c>
-      <c r="E80" s="17" t="s">
-        <v>240</v>
       </c>
       <c r="F80" s="20" t="n">
         <v>2</v>
@@ -7353,13 +7374,13 @@
         <v>194</v>
       </c>
       <c r="J80" s="22" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="K80" s="22" t="s">
         <v>32</v>
       </c>
       <c r="L80" s="22" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="M80" s="17"/>
       <c r="N80" s="17"/>
@@ -7386,10 +7407,10 @@
       <c r="B81" s="37"/>
       <c r="C81" s="26"/>
       <c r="D81" s="17" t="s">
+        <v>242</v>
+      </c>
+      <c r="E81" s="17" t="s">
         <v>243</v>
-      </c>
-      <c r="E81" s="17" t="s">
-        <v>244</v>
       </c>
       <c r="F81" s="38" t="n">
         <v>1</v>
@@ -7404,13 +7425,13 @@
         <v>204</v>
       </c>
       <c r="J81" s="22" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="K81" s="22" t="s">
         <v>32</v>
       </c>
       <c r="L81" s="17" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="M81" s="7"/>
       <c r="N81" s="7"/>
@@ -7437,10 +7458,10 @@
       <c r="B82" s="20"/>
       <c r="C82" s="17"/>
       <c r="D82" s="22" t="s">
+        <v>246</v>
+      </c>
+      <c r="E82" s="17" t="s">
         <v>247</v>
-      </c>
-      <c r="E82" s="17" t="s">
-        <v>248</v>
       </c>
       <c r="F82" s="20" t="n">
         <v>1</v>
@@ -7455,13 +7476,13 @@
         <v>189</v>
       </c>
       <c r="J82" s="22" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="K82" s="22" t="s">
         <v>32</v>
       </c>
       <c r="L82" s="22" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="M82" s="17"/>
       <c r="N82" s="17"/>
@@ -7488,10 +7509,10 @@
       <c r="B83" s="17"/>
       <c r="C83" s="17"/>
       <c r="D83" s="17" t="s">
+        <v>250</v>
+      </c>
+      <c r="E83" s="17" t="s">
         <v>251</v>
-      </c>
-      <c r="E83" s="17" t="s">
-        <v>252</v>
       </c>
       <c r="F83" s="32" t="n">
         <v>2</v>
@@ -7506,13 +7527,13 @@
         <v>189</v>
       </c>
       <c r="J83" s="17" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="K83" s="17" t="s">
         <v>32</v>
       </c>
       <c r="L83" s="17" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="M83" s="17"/>
       <c r="N83" s="17"/>
@@ -7774,10 +7795,10 @@
       <c r="B84" s="20"/>
       <c r="C84" s="17"/>
       <c r="D84" s="22" t="s">
+        <v>254</v>
+      </c>
+      <c r="E84" s="17" t="s">
         <v>255</v>
-      </c>
-      <c r="E84" s="17" t="s">
-        <v>256</v>
       </c>
       <c r="F84" s="20" t="n">
         <v>1</v>
@@ -7789,16 +7810,16 @@
         <v>27</v>
       </c>
       <c r="I84" s="22" t="s">
-        <v>194</v>
+        <v>204</v>
       </c>
       <c r="J84" s="22" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="K84" s="22" t="s">
         <v>32</v>
       </c>
       <c r="L84" s="22" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="M84" s="17"/>
       <c r="N84" s="17"/>
@@ -7825,10 +7846,10 @@
       <c r="B85" s="20"/>
       <c r="C85" s="17"/>
       <c r="D85" s="22" t="s">
+        <v>258</v>
+      </c>
+      <c r="E85" s="17" t="s">
         <v>259</v>
-      </c>
-      <c r="E85" s="17" t="s">
-        <v>260</v>
       </c>
       <c r="F85" s="20" t="n">
         <v>1</v>
@@ -7843,13 +7864,13 @@
         <v>199</v>
       </c>
       <c r="J85" s="22" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="K85" s="22" t="s">
         <v>32</v>
       </c>
       <c r="L85" s="22" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="M85" s="17"/>
       <c r="N85" s="17"/>
@@ -7876,10 +7897,10 @@
       <c r="B86" s="20"/>
       <c r="C86" s="17"/>
       <c r="D86" s="22" t="s">
+        <v>262</v>
+      </c>
+      <c r="E86" s="17" t="s">
         <v>263</v>
-      </c>
-      <c r="E86" s="17" t="s">
-        <v>264</v>
       </c>
       <c r="F86" s="20" t="n">
         <v>1</v>
@@ -7894,13 +7915,13 @@
         <v>209</v>
       </c>
       <c r="J86" s="22" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="K86" s="22" t="s">
         <v>32</v>
       </c>
       <c r="L86" s="22" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="M86" s="17"/>
       <c r="N86" s="17"/>
@@ -7927,10 +7948,10 @@
       <c r="B87" s="20"/>
       <c r="C87" s="17"/>
       <c r="D87" s="22" t="s">
+        <v>266</v>
+      </c>
+      <c r="E87" s="17" t="s">
         <v>267</v>
-      </c>
-      <c r="E87" s="17" t="s">
-        <v>268</v>
       </c>
       <c r="F87" s="20" t="n">
         <v>1</v>
@@ -7945,19 +7966,19 @@
         <v>194</v>
       </c>
       <c r="J87" s="22" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="K87" s="22" t="s">
         <v>32</v>
       </c>
       <c r="L87" s="22" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="M87" s="17" t="s">
         <v>204</v>
       </c>
       <c r="N87" s="17" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="O87" s="17"/>
       <c r="P87" s="17"/>
@@ -7982,10 +8003,10 @@
       <c r="B88" s="17"/>
       <c r="C88" s="17"/>
       <c r="D88" s="17" t="s">
+        <v>271</v>
+      </c>
+      <c r="E88" s="17" t="s">
         <v>272</v>
-      </c>
-      <c r="E88" s="17" t="s">
-        <v>273</v>
       </c>
       <c r="F88" s="32" t="n">
         <v>4</v>
@@ -7997,16 +8018,16 @@
         <v>27</v>
       </c>
       <c r="I88" s="17" t="s">
+        <v>273</v>
+      </c>
+      <c r="J88" s="17" t="s">
         <v>274</v>
-      </c>
-      <c r="J88" s="17" t="s">
-        <v>275</v>
       </c>
       <c r="K88" s="17" t="s">
         <v>32</v>
       </c>
       <c r="L88" s="17" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="M88" s="17"/>
       <c r="N88" s="17"/>
@@ -8268,10 +8289,10 @@
       <c r="B89" s="17"/>
       <c r="C89" s="17"/>
       <c r="D89" s="17" t="s">
+        <v>276</v>
+      </c>
+      <c r="E89" s="17" t="s">
         <v>277</v>
-      </c>
-      <c r="E89" s="17" t="s">
-        <v>278</v>
       </c>
       <c r="F89" s="32" t="n">
         <v>2</v>
@@ -8283,16 +8304,16 @@
         <v>27</v>
       </c>
       <c r="I89" s="43" t="s">
+        <v>278</v>
+      </c>
+      <c r="J89" s="43" t="s">
         <v>279</v>
-      </c>
-      <c r="J89" s="43" t="s">
-        <v>280</v>
       </c>
       <c r="K89" s="43" t="s">
         <v>32</v>
       </c>
       <c r="L89" s="30" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="M89" s="7"/>
       <c r="N89" s="7"/>
@@ -8554,10 +8575,10 @@
       <c r="B90" s="17"/>
       <c r="C90" s="17"/>
       <c r="D90" s="17" t="s">
+        <v>281</v>
+      </c>
+      <c r="E90" s="17" t="s">
         <v>282</v>
-      </c>
-      <c r="E90" s="17" t="s">
-        <v>283</v>
       </c>
       <c r="F90" s="32" t="n">
         <v>2</v>
@@ -8569,22 +8590,22 @@
         <v>27</v>
       </c>
       <c r="I90" s="17" t="s">
+        <v>283</v>
+      </c>
+      <c r="J90" s="17" t="s">
         <v>284</v>
-      </c>
-      <c r="J90" s="17" t="s">
-        <v>285</v>
       </c>
       <c r="K90" s="17" t="s">
         <v>32</v>
       </c>
       <c r="L90" s="17" t="s">
+        <v>285</v>
+      </c>
+      <c r="M90" s="17" t="s">
         <v>286</v>
       </c>
-      <c r="M90" s="17" t="s">
+      <c r="N90" s="17" t="s">
         <v>287</v>
-      </c>
-      <c r="N90" s="17" t="s">
-        <v>288</v>
       </c>
       <c r="O90" s="17"/>
       <c r="P90" s="17"/>
@@ -8844,10 +8865,10 @@
       <c r="B91" s="17"/>
       <c r="C91" s="17"/>
       <c r="D91" s="17" t="s">
+        <v>288</v>
+      </c>
+      <c r="E91" s="17" t="s">
         <v>289</v>
-      </c>
-      <c r="E91" s="17" t="s">
-        <v>290</v>
       </c>
       <c r="F91" s="32" t="n">
         <v>1</v>
@@ -8859,28 +8880,28 @@
         <v>27</v>
       </c>
       <c r="I91" s="17" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="J91" s="17" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K91" s="17" t="s">
         <v>32</v>
       </c>
       <c r="L91" s="17" t="s">
+        <v>291</v>
+      </c>
+      <c r="M91" s="22" t="s">
         <v>292</v>
       </c>
-      <c r="M91" s="22" t="s">
+      <c r="N91" s="17" t="s">
         <v>293</v>
-      </c>
-      <c r="N91" s="17" t="s">
-        <v>294</v>
       </c>
       <c r="O91" s="17" t="s">
         <v>209</v>
       </c>
       <c r="P91" s="17" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="Q91" s="33" t="n">
         <v>0.11</v>
@@ -9138,10 +9159,10 @@
       <c r="B92" s="45"/>
       <c r="C92" s="30"/>
       <c r="D92" s="41" t="s">
+        <v>295</v>
+      </c>
+      <c r="E92" s="30" t="s">
         <v>296</v>
-      </c>
-      <c r="E92" s="30" t="s">
-        <v>297</v>
       </c>
       <c r="F92" s="45" t="n">
         <v>8</v>
@@ -9153,16 +9174,16 @@
         <v>27</v>
       </c>
       <c r="I92" s="41" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="J92" s="41" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="K92" s="41" t="s">
         <v>32</v>
       </c>
       <c r="L92" s="41" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="M92" s="30"/>
       <c r="N92" s="30"/>
@@ -9189,10 +9210,10 @@
       <c r="B93" s="37"/>
       <c r="C93" s="26"/>
       <c r="D93" s="41" t="s">
+        <v>299</v>
+      </c>
+      <c r="E93" s="30" t="s">
         <v>300</v>
-      </c>
-      <c r="E93" s="30" t="s">
-        <v>301</v>
       </c>
       <c r="F93" s="38" t="n">
         <v>2</v>
@@ -9204,16 +9225,16 @@
         <v>27</v>
       </c>
       <c r="I93" s="41" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="J93" s="41" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="K93" s="48" t="s">
         <v>32</v>
       </c>
       <c r="L93" s="30" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="M93" s="49"/>
       <c r="N93" s="7"/>
@@ -9240,10 +9261,10 @@
       <c r="B94" s="20"/>
       <c r="C94" s="17"/>
       <c r="D94" s="22" t="s">
+        <v>303</v>
+      </c>
+      <c r="E94" s="17" t="s">
         <v>304</v>
-      </c>
-      <c r="E94" s="17" t="s">
-        <v>305</v>
       </c>
       <c r="F94" s="20" t="n">
         <v>3</v>
@@ -9255,16 +9276,16 @@
         <v>27</v>
       </c>
       <c r="I94" s="22" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="J94" s="22" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="K94" s="22" t="s">
         <v>32</v>
       </c>
       <c r="L94" s="22" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="M94" s="17"/>
       <c r="N94" s="17"/>
@@ -9291,10 +9312,10 @@
       <c r="B95" s="17"/>
       <c r="C95" s="17"/>
       <c r="D95" s="17" t="s">
+        <v>307</v>
+      </c>
+      <c r="E95" s="17" t="s">
         <v>308</v>
-      </c>
-      <c r="E95" s="17" t="s">
-        <v>309</v>
       </c>
       <c r="F95" s="32" t="n">
         <v>1</v>
@@ -9306,22 +9327,22 @@
         <v>27</v>
       </c>
       <c r="I95" s="17" t="s">
+        <v>309</v>
+      </c>
+      <c r="J95" s="17" t="s">
         <v>310</v>
-      </c>
-      <c r="J95" s="17" t="s">
-        <v>311</v>
       </c>
       <c r="K95" s="17" t="s">
         <v>32</v>
       </c>
       <c r="L95" s="17" t="s">
+        <v>311</v>
+      </c>
+      <c r="M95" s="17" t="s">
+        <v>309</v>
+      </c>
+      <c r="N95" s="17" t="s">
         <v>312</v>
-      </c>
-      <c r="M95" s="17" t="s">
-        <v>310</v>
-      </c>
-      <c r="N95" s="17" t="s">
-        <v>313</v>
       </c>
       <c r="O95" s="17"/>
       <c r="P95" s="17"/>
@@ -9581,10 +9602,10 @@
       <c r="B96" s="20"/>
       <c r="C96" s="17"/>
       <c r="D96" s="22" t="s">
+        <v>313</v>
+      </c>
+      <c r="E96" s="17" t="s">
         <v>314</v>
-      </c>
-      <c r="E96" s="17" t="s">
-        <v>315</v>
       </c>
       <c r="F96" s="20" t="n">
         <v>1</v>
@@ -9596,28 +9617,28 @@
         <v>27</v>
       </c>
       <c r="I96" s="22" t="s">
+        <v>315</v>
+      </c>
+      <c r="J96" s="22" t="s">
         <v>316</v>
-      </c>
-      <c r="J96" s="22" t="s">
-        <v>317</v>
       </c>
       <c r="K96" s="22" t="s">
         <v>32</v>
       </c>
       <c r="L96" s="22" t="s">
+        <v>317</v>
+      </c>
+      <c r="M96" s="17" t="s">
+        <v>286</v>
+      </c>
+      <c r="N96" s="17" t="s">
         <v>318</v>
       </c>
-      <c r="M96" s="17" t="s">
-        <v>287</v>
-      </c>
-      <c r="N96" s="17" t="s">
+      <c r="O96" s="17" t="s">
         <v>319</v>
       </c>
-      <c r="O96" s="17" t="s">
+      <c r="P96" s="17" t="s">
         <v>320</v>
-      </c>
-      <c r="P96" s="17" t="s">
-        <v>321</v>
       </c>
       <c r="Q96" s="15" t="n">
         <v>0.3</v>
@@ -9634,7 +9655,7 @@
         <v>0.181</v>
       </c>
       <c r="U96" s="17" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="97" s="18" customFormat="true" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9642,10 +9663,10 @@
       <c r="B97" s="20"/>
       <c r="C97" s="17"/>
       <c r="D97" s="22" t="s">
+        <v>322</v>
+      </c>
+      <c r="E97" s="17" t="s">
         <v>323</v>
-      </c>
-      <c r="E97" s="17" t="s">
-        <v>324</v>
       </c>
       <c r="F97" s="20" t="n">
         <v>0</v>
@@ -9660,13 +9681,13 @@
         <v>81</v>
       </c>
       <c r="J97" s="22" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="K97" s="22" t="s">
         <v>32</v>
       </c>
       <c r="L97" s="22" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="M97" s="17"/>
       <c r="N97" s="17"/>
@@ -9687,7 +9708,7 @@
         <v>0</v>
       </c>
       <c r="U97" s="17" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="98" s="18" customFormat="true" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9695,10 +9716,10 @@
       <c r="B98" s="20"/>
       <c r="C98" s="17"/>
       <c r="D98" s="22" t="s">
+        <v>327</v>
+      </c>
+      <c r="E98" s="17" t="s">
         <v>328</v>
-      </c>
-      <c r="E98" s="17" t="s">
-        <v>329</v>
       </c>
       <c r="F98" s="20" t="n">
         <v>1</v>
@@ -9713,13 +9734,13 @@
         <v>146</v>
       </c>
       <c r="J98" s="22" t="s">
+        <v>329</v>
+      </c>
+      <c r="K98" s="22" t="s">
         <v>330</v>
       </c>
-      <c r="K98" s="22" t="s">
+      <c r="L98" s="22" t="s">
         <v>331</v>
-      </c>
-      <c r="L98" s="22" t="s">
-        <v>332</v>
       </c>
       <c r="M98" s="17"/>
       <c r="N98" s="17"/>
@@ -9746,10 +9767,10 @@
       <c r="B99" s="20"/>
       <c r="C99" s="17"/>
       <c r="D99" s="22" t="s">
+        <v>332</v>
+      </c>
+      <c r="E99" s="17" t="s">
         <v>333</v>
-      </c>
-      <c r="E99" s="17" t="s">
-        <v>334</v>
       </c>
       <c r="F99" s="20" t="n">
         <v>2</v>
@@ -9764,13 +9785,13 @@
         <v>146</v>
       </c>
       <c r="J99" s="22" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="K99" s="22" t="s">
         <v>32</v>
       </c>
       <c r="L99" s="22" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="M99" s="17"/>
       <c r="N99" s="17"/>
@@ -9797,10 +9818,10 @@
       <c r="B100" s="20"/>
       <c r="C100" s="17"/>
       <c r="D100" s="22" t="s">
+        <v>336</v>
+      </c>
+      <c r="E100" s="17" t="s">
         <v>337</v>
-      </c>
-      <c r="E100" s="17" t="s">
-        <v>338</v>
       </c>
       <c r="F100" s="20" t="n">
         <v>1</v>
@@ -9815,13 +9836,13 @@
         <v>146</v>
       </c>
       <c r="J100" s="22" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="K100" s="22" t="s">
         <v>32</v>
       </c>
       <c r="L100" s="22" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="M100" s="17"/>
       <c r="N100" s="17"/>
@@ -9848,10 +9869,10 @@
       <c r="B101" s="20"/>
       <c r="C101" s="17"/>
       <c r="D101" s="22" t="s">
+        <v>340</v>
+      </c>
+      <c r="E101" s="17" t="s">
         <v>341</v>
-      </c>
-      <c r="E101" s="17" t="s">
-        <v>342</v>
       </c>
       <c r="F101" s="20" t="n">
         <v>1</v>
@@ -9866,13 +9887,13 @@
         <v>146</v>
       </c>
       <c r="J101" s="22" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="K101" s="22" t="s">
         <v>32</v>
       </c>
       <c r="L101" s="22" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="M101" s="17"/>
       <c r="N101" s="17"/>
@@ -9899,10 +9920,10 @@
       <c r="B102" s="20"/>
       <c r="C102" s="17"/>
       <c r="D102" s="22" t="s">
+        <v>344</v>
+      </c>
+      <c r="E102" s="17" t="s">
         <v>345</v>
-      </c>
-      <c r="E102" s="17" t="s">
-        <v>346</v>
       </c>
       <c r="F102" s="20" t="n">
         <v>1</v>
@@ -9914,16 +9935,16 @@
         <v>27</v>
       </c>
       <c r="I102" s="22" t="s">
+        <v>346</v>
+      </c>
+      <c r="J102" s="22" t="s">
         <v>347</v>
-      </c>
-      <c r="J102" s="22" t="s">
-        <v>348</v>
       </c>
       <c r="K102" s="22" t="s">
         <v>32</v>
       </c>
       <c r="L102" s="22" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="M102" s="17"/>
       <c r="N102" s="17"/>
@@ -9950,10 +9971,10 @@
       <c r="B103" s="20"/>
       <c r="C103" s="17"/>
       <c r="D103" s="22" t="s">
+        <v>349</v>
+      </c>
+      <c r="E103" s="17" t="s">
         <v>350</v>
-      </c>
-      <c r="E103" s="17" t="s">
-        <v>351</v>
       </c>
       <c r="F103" s="20" t="n">
         <v>2</v>
@@ -9965,16 +9986,16 @@
         <v>27</v>
       </c>
       <c r="I103" s="22" t="s">
+        <v>351</v>
+      </c>
+      <c r="J103" s="22" t="s">
         <v>352</v>
-      </c>
-      <c r="J103" s="22" t="s">
-        <v>353</v>
       </c>
       <c r="K103" s="22" t="s">
         <v>32</v>
       </c>
       <c r="L103" s="22" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="M103" s="17"/>
       <c r="N103" s="17"/>
@@ -10001,10 +10022,10 @@
       <c r="B104" s="20"/>
       <c r="C104" s="17"/>
       <c r="D104" s="22" t="s">
+        <v>354</v>
+      </c>
+      <c r="E104" s="17" t="s">
         <v>355</v>
-      </c>
-      <c r="E104" s="17" t="s">
-        <v>356</v>
       </c>
       <c r="F104" s="20" t="n">
         <v>1</v>
@@ -10016,25 +10037,25 @@
         <v>27</v>
       </c>
       <c r="I104" s="22" t="s">
+        <v>356</v>
+      </c>
+      <c r="J104" s="22" t="s">
         <v>357</v>
-      </c>
-      <c r="J104" s="22" t="s">
-        <v>358</v>
       </c>
       <c r="K104" s="22" t="s">
         <v>32</v>
       </c>
       <c r="L104" s="22" t="s">
+        <v>358</v>
+      </c>
+      <c r="M104" s="17" t="s">
         <v>359</v>
       </c>
-      <c r="M104" s="17" t="s">
+      <c r="N104" s="17" t="s">
         <v>360</v>
       </c>
-      <c r="N104" s="17" t="s">
+      <c r="O104" s="17" t="s">
         <v>361</v>
-      </c>
-      <c r="O104" s="17" t="s">
-        <v>362</v>
       </c>
       <c r="P104" s="17" t="n">
         <v>74404054150</v>
@@ -10060,10 +10081,10 @@
       <c r="B105" s="17"/>
       <c r="C105" s="17"/>
       <c r="D105" s="17" t="s">
+        <v>362</v>
+      </c>
+      <c r="E105" s="17" t="s">
         <v>363</v>
-      </c>
-      <c r="E105" s="17" t="s">
-        <v>364</v>
       </c>
       <c r="F105" s="32" t="n">
         <v>4</v>
@@ -10075,28 +10096,28 @@
         <v>27</v>
       </c>
       <c r="I105" s="22" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="J105" s="17" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="K105" s="17" t="s">
         <v>32</v>
       </c>
       <c r="L105" s="17" t="s">
+        <v>365</v>
+      </c>
+      <c r="M105" s="17" t="s">
+        <v>283</v>
+      </c>
+      <c r="N105" s="17" t="s">
         <v>366</v>
       </c>
-      <c r="M105" s="17" t="s">
-        <v>284</v>
-      </c>
-      <c r="N105" s="17" t="s">
+      <c r="O105" s="22" t="s">
         <v>367</v>
       </c>
-      <c r="O105" s="22" t="s">
+      <c r="P105" s="17" t="s">
         <v>368</v>
-      </c>
-      <c r="P105" s="17" t="s">
-        <v>369</v>
       </c>
       <c r="Q105" s="33" t="n">
         <v>0.12</v>
@@ -10354,10 +10375,10 @@
       <c r="B106" s="20"/>
       <c r="C106" s="17"/>
       <c r="D106" s="22" t="s">
+        <v>369</v>
+      </c>
+      <c r="E106" s="17" t="s">
         <v>370</v>
-      </c>
-      <c r="E106" s="17" t="s">
-        <v>371</v>
       </c>
       <c r="F106" s="20" t="n">
         <v>4</v>
@@ -10369,28 +10390,28 @@
         <v>27</v>
       </c>
       <c r="I106" s="22" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="J106" s="22" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="K106" s="22" t="s">
         <v>32</v>
       </c>
       <c r="L106" s="22" t="s">
+        <v>372</v>
+      </c>
+      <c r="M106" s="22" t="s">
         <v>373</v>
       </c>
-      <c r="M106" s="22" t="s">
+      <c r="N106" s="17" t="s">
         <v>374</v>
       </c>
-      <c r="N106" s="17" t="s">
+      <c r="O106" s="17" t="s">
+        <v>286</v>
+      </c>
+      <c r="P106" s="17" t="s">
         <v>375</v>
-      </c>
-      <c r="O106" s="17" t="s">
-        <v>287</v>
-      </c>
-      <c r="P106" s="17" t="s">
-        <v>376</v>
       </c>
       <c r="Q106" s="15" t="n">
         <v>0.12</v>
@@ -10413,10 +10434,10 @@
       <c r="B107" s="20"/>
       <c r="C107" s="17"/>
       <c r="D107" s="22" t="s">
+        <v>376</v>
+      </c>
+      <c r="E107" s="17" t="s">
         <v>377</v>
-      </c>
-      <c r="E107" s="17" t="s">
-        <v>378</v>
       </c>
       <c r="F107" s="20" t="n">
         <v>1</v>
@@ -10428,16 +10449,16 @@
         <v>27</v>
       </c>
       <c r="I107" s="22" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="J107" s="22" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="K107" s="22" t="s">
         <v>32</v>
       </c>
       <c r="L107" s="22" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="M107" s="17"/>
       <c r="N107" s="17"/>
@@ -10464,10 +10485,10 @@
       <c r="B108" s="17"/>
       <c r="C108" s="17"/>
       <c r="D108" s="17" t="s">
+        <v>380</v>
+      </c>
+      <c r="E108" s="17" t="s">
         <v>381</v>
-      </c>
-      <c r="E108" s="17" t="s">
-        <v>382</v>
       </c>
       <c r="F108" s="32" t="n">
         <v>2</v>
@@ -10479,16 +10500,16 @@
         <v>27</v>
       </c>
       <c r="I108" s="17" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="J108" s="17" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="K108" s="17" t="s">
         <v>32</v>
       </c>
       <c r="L108" s="17" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="M108" s="17"/>
       <c r="N108" s="17"/>
@@ -10750,10 +10771,10 @@
       <c r="B109" s="17"/>
       <c r="C109" s="17"/>
       <c r="D109" s="17" t="s">
+        <v>384</v>
+      </c>
+      <c r="E109" s="17" t="s">
         <v>385</v>
-      </c>
-      <c r="E109" s="17" t="s">
-        <v>386</v>
       </c>
       <c r="F109" s="32" t="n">
         <v>2</v>
@@ -10765,16 +10786,16 @@
         <v>27</v>
       </c>
       <c r="I109" s="17" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="J109" s="17" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="K109" s="17" t="s">
         <v>32</v>
       </c>
       <c r="L109" s="17" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="M109" s="17"/>
       <c r="N109" s="17"/>
@@ -11036,10 +11057,10 @@
       <c r="B110" s="17"/>
       <c r="C110" s="17"/>
       <c r="D110" s="17" t="s">
+        <v>388</v>
+      </c>
+      <c r="E110" s="17" t="s">
         <v>389</v>
-      </c>
-      <c r="E110" s="17" t="s">
-        <v>390</v>
       </c>
       <c r="F110" s="32" t="n">
         <v>1</v>
@@ -11051,28 +11072,28 @@
         <v>27</v>
       </c>
       <c r="I110" s="17" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="J110" s="17" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="K110" s="17" t="s">
         <v>32</v>
       </c>
       <c r="L110" s="17" t="s">
+        <v>391</v>
+      </c>
+      <c r="M110" s="17" t="s">
+        <v>315</v>
+      </c>
+      <c r="N110" s="17" t="s">
         <v>392</v>
       </c>
-      <c r="M110" s="17" t="s">
-        <v>316</v>
-      </c>
-      <c r="N110" s="17" t="s">
+      <c r="O110" s="22" t="s">
         <v>393</v>
       </c>
-      <c r="O110" s="22" t="s">
+      <c r="P110" s="17" t="s">
         <v>394</v>
-      </c>
-      <c r="P110" s="17" t="s">
-        <v>395</v>
       </c>
       <c r="Q110" s="33" t="n">
         <v>0.44</v>
@@ -11330,10 +11351,10 @@
       <c r="B111" s="8"/>
       <c r="C111" s="10"/>
       <c r="D111" s="22" t="s">
+        <v>395</v>
+      </c>
+      <c r="E111" s="30" t="s">
         <v>396</v>
-      </c>
-      <c r="E111" s="30" t="s">
-        <v>397</v>
       </c>
       <c r="F111" s="20" t="n">
         <v>1</v>
@@ -11345,16 +11366,16 @@
         <v>27</v>
       </c>
       <c r="I111" s="22" t="s">
+        <v>397</v>
+      </c>
+      <c r="J111" s="22" t="s">
         <v>398</v>
-      </c>
-      <c r="J111" s="22" t="s">
-        <v>399</v>
       </c>
       <c r="K111" s="53" t="s">
         <v>32</v>
       </c>
       <c r="L111" s="17" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="M111" s="54"/>
       <c r="N111" s="17"/>
@@ -11381,10 +11402,10 @@
       <c r="B112" s="20"/>
       <c r="C112" s="17"/>
       <c r="D112" s="22" t="s">
+        <v>400</v>
+      </c>
+      <c r="E112" s="17" t="s">
         <v>401</v>
-      </c>
-      <c r="E112" s="17" t="s">
-        <v>402</v>
       </c>
       <c r="F112" s="20" t="n">
         <v>2</v>
@@ -11396,16 +11417,16 @@
         <v>27</v>
       </c>
       <c r="I112" s="22" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="J112" s="22" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="K112" s="22" t="s">
         <v>32</v>
       </c>
       <c r="L112" s="22" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="M112" s="17"/>
       <c r="N112" s="17"/>
@@ -11432,10 +11453,10 @@
       <c r="B113" s="20"/>
       <c r="C113" s="17"/>
       <c r="D113" s="22" t="s">
+        <v>404</v>
+      </c>
+      <c r="E113" s="17" t="s">
         <v>405</v>
-      </c>
-      <c r="E113" s="17" t="s">
-        <v>406</v>
       </c>
       <c r="F113" s="20" t="n">
         <v>2</v>
@@ -11447,19 +11468,23 @@
         <v>27</v>
       </c>
       <c r="I113" s="22" t="s">
+        <v>406</v>
+      </c>
+      <c r="J113" s="22" t="s">
         <v>407</v>
-      </c>
-      <c r="J113" s="22" t="s">
-        <v>408</v>
       </c>
       <c r="K113" s="22" t="s">
         <v>32</v>
       </c>
       <c r="L113" s="22" t="s">
+        <v>408</v>
+      </c>
+      <c r="M113" s="17" t="s">
         <v>409</v>
       </c>
-      <c r="M113" s="17"/>
-      <c r="N113" s="17"/>
+      <c r="N113" s="17" t="s">
+        <v>410</v>
+      </c>
       <c r="O113" s="17"/>
       <c r="P113" s="17"/>
       <c r="Q113" s="15" t="n">
@@ -11483,10 +11508,10 @@
       <c r="B114" s="20"/>
       <c r="C114" s="17"/>
       <c r="D114" s="22" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="E114" s="17" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="F114" s="20" t="n">
         <v>1</v>
@@ -11498,16 +11523,16 @@
         <v>27</v>
       </c>
       <c r="I114" s="22" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="J114" s="22" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="K114" s="22" t="s">
         <v>32</v>
       </c>
       <c r="L114" s="22" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="M114" s="17"/>
       <c r="N114" s="17"/>
@@ -11528,10 +11553,10 @@
       <c r="B115" s="8"/>
       <c r="C115" s="10"/>
       <c r="D115" s="22" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="E115" s="30" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="F115" s="20" t="n">
         <v>6</v>
@@ -11543,16 +11568,16 @@
         <v>27</v>
       </c>
       <c r="I115" s="22" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="J115" s="22" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="K115" s="53" t="s">
         <v>32</v>
       </c>
       <c r="L115" s="17" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="M115" s="54"/>
       <c r="N115" s="17"/>
@@ -11579,10 +11604,10 @@
       <c r="B116" s="8"/>
       <c r="C116" s="10"/>
       <c r="D116" s="22" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="E116" s="30" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="F116" s="20" t="n">
         <v>7</v>
@@ -11594,16 +11619,16 @@
         <v>27</v>
       </c>
       <c r="I116" s="22" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="J116" s="22" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="K116" s="53" t="s">
         <v>32</v>
       </c>
       <c r="L116" s="17" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="M116" s="54"/>
       <c r="N116" s="17"/>
@@ -11630,10 +11655,10 @@
       <c r="B117" s="8"/>
       <c r="C117" s="10"/>
       <c r="D117" s="22" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="E117" s="30" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="F117" s="20" t="n">
         <v>6</v>
@@ -11645,16 +11670,16 @@
         <v>27</v>
       </c>
       <c r="I117" s="22" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="J117" s="22" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="K117" s="53" t="s">
         <v>32</v>
       </c>
       <c r="L117" s="17" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="M117" s="54"/>
       <c r="N117" s="17"/>
@@ -11681,10 +11706,10 @@
       <c r="B118" s="8"/>
       <c r="C118" s="10"/>
       <c r="D118" s="22" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="E118" s="30" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="F118" s="20" t="n">
         <v>4</v>
@@ -11696,16 +11721,16 @@
         <v>27</v>
       </c>
       <c r="I118" s="22" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="J118" s="22" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="K118" s="53" t="s">
         <v>32</v>
       </c>
       <c r="L118" s="17" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="M118" s="54"/>
       <c r="N118" s="17"/>
@@ -11732,10 +11757,10 @@
       <c r="B119" s="8"/>
       <c r="C119" s="10"/>
       <c r="D119" s="22" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E119" s="30" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="F119" s="20" t="n">
         <v>2</v>
@@ -11747,16 +11772,16 @@
         <v>27</v>
       </c>
       <c r="I119" s="22" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="J119" s="22" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="K119" s="53" t="s">
         <v>32</v>
       </c>
       <c r="L119" s="17" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="M119" s="54"/>
       <c r="N119" s="17"/>
@@ -11783,10 +11808,10 @@
       <c r="B120" s="8"/>
       <c r="C120" s="10"/>
       <c r="D120" s="22" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="E120" s="30" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="F120" s="20" t="n">
         <v>4</v>
@@ -11798,16 +11823,16 @@
         <v>27</v>
       </c>
       <c r="I120" s="22" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="J120" s="22" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="K120" s="53" t="s">
         <v>32</v>
       </c>
       <c r="L120" s="17" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="M120" s="54"/>
       <c r="N120" s="17"/>
@@ -11834,10 +11859,10 @@
       <c r="B121" s="8"/>
       <c r="C121" s="10"/>
       <c r="D121" s="22" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="E121" s="30" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="F121" s="20" t="n">
         <v>2</v>
@@ -11852,13 +11877,13 @@
         <v>209</v>
       </c>
       <c r="J121" s="22" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="K121" s="53" t="s">
         <v>32</v>
       </c>
       <c r="L121" s="17" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="M121" s="54"/>
       <c r="N121" s="17"/>
@@ -11885,10 +11910,10 @@
       <c r="B122" s="8"/>
       <c r="C122" s="10"/>
       <c r="D122" s="22" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="E122" s="30" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="F122" s="20" t="n">
         <v>1</v>
@@ -11900,16 +11925,16 @@
         <v>27</v>
       </c>
       <c r="I122" s="22" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="J122" s="22" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="K122" s="53" t="s">
         <v>32</v>
       </c>
       <c r="L122" s="17" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="M122" s="54"/>
       <c r="N122" s="17"/>
@@ -11936,10 +11961,10 @@
       <c r="B123" s="8"/>
       <c r="C123" s="10"/>
       <c r="D123" s="22" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E123" s="30" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="F123" s="20" t="n">
         <v>1</v>
@@ -11951,16 +11976,16 @@
         <v>27</v>
       </c>
       <c r="I123" s="22" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="J123" s="22" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="K123" s="53" t="s">
         <v>32</v>
       </c>
       <c r="L123" s="17" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="M123" s="54"/>
       <c r="N123" s="17"/>
@@ -11987,10 +12012,10 @@
       <c r="B124" s="8"/>
       <c r="C124" s="10"/>
       <c r="D124" s="22" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="E124" s="30" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="F124" s="20" t="n">
         <v>1</v>
@@ -12002,16 +12027,16 @@
         <v>27</v>
       </c>
       <c r="I124" s="22" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="J124" s="22" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="K124" s="53" t="s">
         <v>32</v>
       </c>
       <c r="L124" s="17" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="M124" s="54"/>
       <c r="N124" s="17"/>
@@ -12038,10 +12063,10 @@
       <c r="B125" s="8"/>
       <c r="C125" s="10"/>
       <c r="D125" s="22" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="E125" s="30" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="F125" s="20" t="n">
         <v>8</v>
@@ -12053,16 +12078,16 @@
         <v>27</v>
       </c>
       <c r="I125" s="22" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="J125" s="22" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="K125" s="53" t="s">
         <v>32</v>
       </c>
       <c r="L125" s="17" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="M125" s="54"/>
       <c r="N125" s="17"/>
@@ -12089,10 +12114,10 @@
       <c r="B126" s="8"/>
       <c r="C126" s="10"/>
       <c r="D126" s="22" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="E126" s="30" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="F126" s="20" t="n">
         <v>1</v>
@@ -12104,16 +12129,16 @@
         <v>27</v>
       </c>
       <c r="I126" s="22" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="J126" s="22" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="K126" s="53" t="s">
         <v>32</v>
       </c>
       <c r="L126" s="17" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="M126" s="54"/>
       <c r="N126" s="17"/>
@@ -12140,10 +12165,10 @@
       <c r="B127" s="8"/>
       <c r="C127" s="10"/>
       <c r="D127" s="22" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="E127" s="30" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="F127" s="20" t="n">
         <v>5</v>
@@ -12155,16 +12180,16 @@
         <v>27</v>
       </c>
       <c r="I127" s="22" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="J127" s="22" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="K127" s="53" t="s">
         <v>32</v>
       </c>
       <c r="L127" s="17" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="M127" s="54"/>
       <c r="N127" s="17"/>
@@ -12191,10 +12216,10 @@
       <c r="B128" s="8"/>
       <c r="C128" s="10"/>
       <c r="D128" s="22" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="E128" s="30" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="F128" s="20" t="n">
         <v>2</v>
@@ -12206,16 +12231,16 @@
         <v>27</v>
       </c>
       <c r="I128" s="22" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="J128" s="22" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="K128" s="53" t="s">
         <v>32</v>
       </c>
       <c r="L128" s="17" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="M128" s="54"/>
       <c r="N128" s="17"/>
@@ -12242,10 +12267,10 @@
       <c r="B129" s="8"/>
       <c r="C129" s="10"/>
       <c r="D129" s="22" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="E129" s="30" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="F129" s="20" t="n">
         <v>1</v>
@@ -12257,16 +12282,16 @@
         <v>27</v>
       </c>
       <c r="I129" s="22" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="J129" s="22" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="K129" s="53" t="s">
         <v>32</v>
       </c>
       <c r="L129" s="17" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="M129" s="54"/>
       <c r="N129" s="17"/>
@@ -12293,10 +12318,10 @@
       <c r="B130" s="8"/>
       <c r="C130" s="10"/>
       <c r="D130" s="22" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="E130" s="30" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="F130" s="20" t="n">
         <v>2</v>
@@ -12308,16 +12333,16 @@
         <v>27</v>
       </c>
       <c r="I130" s="22" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="J130" s="22" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="K130" s="53" t="s">
         <v>32</v>
       </c>
       <c r="L130" s="17" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="M130" s="54"/>
       <c r="N130" s="17"/>
@@ -12344,10 +12369,10 @@
       <c r="B131" s="8"/>
       <c r="C131" s="10"/>
       <c r="D131" s="22" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="E131" s="30" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="F131" s="20" t="n">
         <v>2</v>
@@ -12359,16 +12384,16 @@
         <v>27</v>
       </c>
       <c r="I131" s="22" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="J131" s="22" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="K131" s="53" t="s">
         <v>32</v>
       </c>
       <c r="L131" s="17" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="M131" s="54"/>
       <c r="N131" s="17"/>
@@ -12395,10 +12420,10 @@
       <c r="B132" s="8"/>
       <c r="C132" s="10"/>
       <c r="D132" s="22" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="E132" s="30" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="F132" s="20" t="n">
         <v>2</v>
@@ -12410,16 +12435,16 @@
         <v>27</v>
       </c>
       <c r="I132" s="22" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="J132" s="22" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="K132" s="53" t="s">
         <v>32</v>
       </c>
       <c r="L132" s="17" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="M132" s="54"/>
       <c r="N132" s="17"/>
@@ -12446,10 +12471,10 @@
       <c r="B133" s="8"/>
       <c r="C133" s="10"/>
       <c r="D133" s="22" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="E133" s="30" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="F133" s="20" t="n">
         <v>2</v>
@@ -12461,16 +12486,16 @@
         <v>27</v>
       </c>
       <c r="I133" s="22" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="J133" s="22" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="K133" s="53" t="s">
         <v>32</v>
       </c>
       <c r="L133" s="17" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="M133" s="54"/>
       <c r="N133" s="17"/>
@@ -12497,10 +12522,10 @@
       <c r="B134" s="8"/>
       <c r="C134" s="10"/>
       <c r="D134" s="22" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="E134" s="30" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="F134" s="20" t="n">
         <v>2</v>
@@ -12512,16 +12537,16 @@
         <v>27</v>
       </c>
       <c r="I134" s="22" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="J134" s="22" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="K134" s="53" t="s">
         <v>32</v>
       </c>
       <c r="L134" s="17" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="M134" s="54"/>
       <c r="N134" s="17"/>
@@ -12548,10 +12573,10 @@
       <c r="B135" s="8"/>
       <c r="C135" s="10"/>
       <c r="D135" s="22" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="E135" s="30" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="F135" s="20" t="n">
         <v>2</v>
@@ -12563,16 +12588,16 @@
         <v>27</v>
       </c>
       <c r="I135" s="22" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="J135" s="22" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="K135" s="53" t="s">
         <v>32</v>
       </c>
       <c r="L135" s="17" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="M135" s="54"/>
       <c r="N135" s="17"/>
@@ -12599,10 +12624,10 @@
       <c r="B136" s="8"/>
       <c r="C136" s="10"/>
       <c r="D136" s="22" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="E136" s="30" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="F136" s="20" t="n">
         <v>2</v>
@@ -12614,16 +12639,16 @@
         <v>27</v>
       </c>
       <c r="I136" s="22" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="J136" s="22" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="K136" s="53" t="s">
         <v>32</v>
       </c>
       <c r="L136" s="17" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="M136" s="54"/>
       <c r="N136" s="17"/>
@@ -12650,10 +12675,10 @@
       <c r="B137" s="8"/>
       <c r="C137" s="10"/>
       <c r="D137" s="22" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="E137" s="30" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="F137" s="20" t="n">
         <v>1</v>
@@ -12665,16 +12690,16 @@
         <v>27</v>
       </c>
       <c r="I137" s="22" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="J137" s="22" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="K137" s="53" t="s">
         <v>32</v>
       </c>
       <c r="L137" s="17" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="M137" s="54"/>
       <c r="N137" s="17"/>
@@ -12701,10 +12726,10 @@
       <c r="B138" s="8"/>
       <c r="C138" s="10"/>
       <c r="D138" s="22" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="E138" s="30" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="F138" s="20" t="n">
         <v>1</v>
@@ -12716,16 +12741,16 @@
         <v>27</v>
       </c>
       <c r="I138" s="22" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="J138" s="22" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="K138" s="53" t="s">
         <v>32</v>
       </c>
       <c r="L138" s="17" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="M138" s="54"/>
       <c r="N138" s="17"/>
@@ -12752,10 +12777,10 @@
       <c r="B139" s="8"/>
       <c r="C139" s="10"/>
       <c r="D139" s="22" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="E139" s="30" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="F139" s="20" t="n">
         <v>0</v>
@@ -12767,16 +12792,16 @@
         <v>27</v>
       </c>
       <c r="I139" s="22" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="J139" s="22" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="K139" s="53" t="s">
         <v>32</v>
       </c>
       <c r="L139" s="17" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="M139" s="54"/>
       <c r="N139" s="17"/>
@@ -12797,7 +12822,7 @@
         <v>0</v>
       </c>
       <c r="U139" s="59" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="140" s="18" customFormat="true" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12807,10 +12832,10 @@
         <v>43</v>
       </c>
       <c r="D140" s="22" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="E140" s="30" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="F140" s="20" t="n">
         <v>1</v>
@@ -12822,16 +12847,16 @@
         <v>23</v>
       </c>
       <c r="I140" s="22" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="J140" s="22" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="K140" s="53" t="s">
         <v>32</v>
       </c>
       <c r="L140" s="17" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="M140" s="54"/>
       <c r="N140" s="17"/>
@@ -12860,10 +12885,10 @@
         <v>43</v>
       </c>
       <c r="D141" s="22" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="E141" s="30" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="F141" s="20" t="n">
         <v>1</v>
@@ -12875,16 +12900,16 @@
         <v>23</v>
       </c>
       <c r="I141" s="22" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="J141" s="22" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="K141" s="53" t="s">
         <v>32</v>
       </c>
       <c r="L141" s="17" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="M141" s="54"/>
       <c r="N141" s="17"/>
@@ -12913,10 +12938,10 @@
         <v>43</v>
       </c>
       <c r="D142" s="22" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="E142" s="30" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="F142" s="20" t="n">
         <v>2</v>
@@ -12928,16 +12953,16 @@
         <v>23</v>
       </c>
       <c r="I142" s="22" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="J142" s="22" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="K142" s="53" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="L142" s="17" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="M142" s="54"/>
       <c r="N142" s="17"/>
@@ -12964,10 +12989,10 @@
       <c r="B143" s="8"/>
       <c r="C143" s="10"/>
       <c r="D143" s="22" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="E143" s="30" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="F143" s="20" t="n">
         <v>2</v>
@@ -12979,28 +13004,28 @@
         <v>27</v>
       </c>
       <c r="I143" s="22" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="J143" s="22" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="K143" s="53" t="s">
         <v>32</v>
       </c>
       <c r="L143" s="17" t="s">
+        <v>532</v>
+      </c>
+      <c r="M143" s="54" t="s">
+        <v>533</v>
+      </c>
+      <c r="N143" s="17" t="s">
+        <v>534</v>
+      </c>
+      <c r="O143" s="17" t="s">
+        <v>535</v>
+      </c>
+      <c r="P143" s="17" t="s">
         <v>531</v>
-      </c>
-      <c r="M143" s="54" t="s">
-        <v>532</v>
-      </c>
-      <c r="N143" s="17" t="s">
-        <v>533</v>
-      </c>
-      <c r="O143" s="17" t="s">
-        <v>534</v>
-      </c>
-      <c r="P143" s="17" t="s">
-        <v>530</v>
       </c>
       <c r="Q143" s="55" t="n">
         <v>0.18</v>
@@ -13023,10 +13048,10 @@
       <c r="B144" s="8"/>
       <c r="C144" s="10"/>
       <c r="D144" s="22" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="E144" s="30" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="F144" s="20" t="n">
         <v>1</v>
@@ -13038,16 +13063,16 @@
         <v>27</v>
       </c>
       <c r="I144" s="22" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="J144" s="22" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="K144" s="53" t="s">
         <v>32</v>
       </c>
       <c r="L144" s="17" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="M144" s="54"/>
       <c r="N144" s="17"/>
@@ -13074,10 +13099,10 @@
       <c r="B145" s="8"/>
       <c r="C145" s="10"/>
       <c r="D145" s="22" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="E145" s="30" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F145" s="20" t="n">
         <v>1</v>
@@ -13089,28 +13114,28 @@
         <v>27</v>
       </c>
       <c r="I145" s="22" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="J145" s="22" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="K145" s="53" t="s">
         <v>32</v>
       </c>
       <c r="L145" s="17" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="M145" s="60" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="N145" s="17" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="O145" s="17" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="P145" s="17" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="Q145" s="55" t="n">
         <v>0.38</v>
@@ -13133,10 +13158,10 @@
       <c r="B146" s="20"/>
       <c r="C146" s="17"/>
       <c r="D146" s="22" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="E146" s="17" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="F146" s="20" t="n">
         <v>2</v>
@@ -13148,16 +13173,16 @@
         <v>27</v>
       </c>
       <c r="I146" s="22" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="J146" s="22" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="K146" s="22" t="s">
         <v>32</v>
       </c>
       <c r="L146" s="22" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="M146" s="17"/>
       <c r="N146" s="17"/>
@@ -13184,10 +13209,10 @@
       <c r="B147" s="20"/>
       <c r="C147" s="17"/>
       <c r="D147" s="22" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="E147" s="17" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="F147" s="20" t="n">
         <v>1</v>
@@ -13199,16 +13224,16 @@
         <v>27</v>
       </c>
       <c r="I147" s="22" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="J147" s="22" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="K147" s="22" t="s">
         <v>32</v>
       </c>
       <c r="L147" s="22" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="M147" s="17"/>
       <c r="N147" s="17"/>
@@ -13235,10 +13260,10 @@
       <c r="B148" s="8"/>
       <c r="C148" s="10"/>
       <c r="D148" s="22" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="E148" s="30" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="F148" s="20" t="n">
         <v>2</v>
@@ -13250,16 +13275,16 @@
         <v>27</v>
       </c>
       <c r="I148" s="22" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="J148" s="22" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="K148" s="53" t="s">
         <v>32</v>
       </c>
       <c r="L148" s="17" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="M148" s="54"/>
       <c r="N148" s="17"/>
@@ -13286,10 +13311,10 @@
       <c r="B149" s="20"/>
       <c r="C149" s="17"/>
       <c r="D149" s="22" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="E149" s="17" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="F149" s="20" t="n">
         <v>1</v>
@@ -13301,28 +13326,28 @@
         <v>27</v>
       </c>
       <c r="I149" s="22" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="J149" s="22" t="s">
+        <v>564</v>
+      </c>
+      <c r="K149" s="22" t="s">
+        <v>330</v>
+      </c>
+      <c r="L149" s="22" t="s">
+        <v>565</v>
+      </c>
+      <c r="M149" s="17" t="s">
         <v>563</v>
       </c>
-      <c r="K149" s="22" t="s">
-        <v>331</v>
-      </c>
-      <c r="L149" s="22" t="s">
-        <v>564</v>
-      </c>
-      <c r="M149" s="17" t="s">
-        <v>562</v>
-      </c>
       <c r="N149" s="17" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="O149" s="17" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="P149" s="17" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="Q149" s="15" t="n">
         <v>0.66</v>
@@ -13345,10 +13370,10 @@
       <c r="B150" s="20"/>
       <c r="C150" s="17"/>
       <c r="D150" s="22" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="E150" s="17" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="F150" s="20" t="n">
         <v>1</v>
@@ -13360,22 +13385,22 @@
         <v>27</v>
       </c>
       <c r="I150" s="22" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="J150" s="22" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="K150" s="22" t="s">
         <v>32</v>
       </c>
       <c r="L150" s="22" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="M150" s="17" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="N150" s="17" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="O150" s="17"/>
       <c r="P150" s="17"/>
@@ -13400,10 +13425,10 @@
       <c r="B151" s="20"/>
       <c r="C151" s="17"/>
       <c r="D151" s="22" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="E151" s="17" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="F151" s="20" t="n">
         <v>1</v>
@@ -13415,16 +13440,16 @@
         <v>27</v>
       </c>
       <c r="I151" s="22" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="J151" s="22" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="K151" s="22" t="s">
         <v>32</v>
       </c>
       <c r="L151" s="22" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="M151" s="17"/>
       <c r="N151" s="17"/>
@@ -13451,10 +13476,10 @@
       <c r="B152" s="20"/>
       <c r="C152" s="17"/>
       <c r="D152" s="22" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="E152" s="17" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="F152" s="20" t="n">
         <v>1</v>
@@ -13466,16 +13491,16 @@
         <v>27</v>
       </c>
       <c r="I152" s="22" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="J152" s="22" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="K152" s="22" t="s">
         <v>32</v>
       </c>
       <c r="L152" s="22" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="M152" s="17"/>
       <c r="N152" s="17"/>
@@ -13502,10 +13527,10 @@
       <c r="B153" s="20"/>
       <c r="C153" s="17"/>
       <c r="D153" s="22" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="E153" s="17" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="F153" s="20" t="n">
         <v>1</v>
@@ -13517,16 +13542,16 @@
         <v>27</v>
       </c>
       <c r="I153" s="22" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="J153" s="22" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="K153" s="22" t="s">
         <v>32</v>
       </c>
       <c r="L153" s="22" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="M153" s="17"/>
       <c r="N153" s="17"/>
@@ -13555,7 +13580,7 @@
         <v>43</v>
       </c>
       <c r="D154" s="22" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="E154" s="17"/>
       <c r="F154" s="20" t="n">
@@ -13568,13 +13593,13 @@
         <v>23</v>
       </c>
       <c r="I154" s="22" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="J154" s="22" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="K154" s="22" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="L154" s="61"/>
       <c r="M154" s="17"/>
@@ -13596,7 +13621,7 @@
         <v>36</v>
       </c>
       <c r="U154" s="57" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13613,31 +13638,43 @@
       <c r="G157" s="65"/>
       <c r="H157" s="65"/>
       <c r="P157" s="66" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="Q157" s="15"/>
       <c r="R157" s="67" t="n">
         <f aca="false">SUM(R3:R154)</f>
-        <v>193.2295</v>
+        <v>193.1295</v>
       </c>
       <c r="S157" s="68"/>
       <c r="T157" s="69" t="n">
         <f aca="false">SUM(T3:T154)</f>
-        <v>120.91215</v>
+        <v>121.17215</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D158" s="1" t="s">
+        <v>592</v>
+      </c>
+      <c r="I158" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="J158" s="1" t="s">
+        <v>593</v>
+      </c>
+      <c r="K158" s="1" t="s">
+        <v>594</v>
+      </c>
       <c r="Q158" s="63"/>
       <c r="T158" s="64"/>
     </row>
     <row r="159" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J159" s="1" t="s">
+        <v>595</v>
+      </c>
       <c r="Q159" s="63"/>
       <c r="T159" s="64"/>
     </row>
     <row r="160" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A160" s="70" t="s">
-        <v>591</v>
-      </c>
       <c r="Q160" s="63"/>
       <c r="T160" s="64"/>
     </row>
@@ -13646,12 +13683,33 @@
       <c r="T161" s="64"/>
     </row>
     <row r="162" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D162" s="1" t="s">
+        <v>596</v>
+      </c>
+      <c r="I162" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="J162" s="1" t="s">
+        <v>597</v>
+      </c>
       <c r="Q162" s="63"/>
       <c r="T162" s="64"/>
     </row>
-    <row r="1048555" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048556" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048557" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="163" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A163" s="70" t="s">
+        <v>598</v>
+      </c>
+      <c r="Q163" s="63"/>
+      <c r="T163" s="64"/>
+    </row>
+    <row r="164" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Q164" s="63"/>
+      <c r="T164" s="64"/>
+    </row>
+    <row r="165" customFormat="false" ht="14.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Q165" s="63"/>
+      <c r="T165" s="64"/>
+    </row>
     <row r="1048558" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048559" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048560" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>